<commit_message>
# fix AI's error and update README
</commit_message>
<xml_diff>
--- a/index.xlsx
+++ b/index.xlsx
@@ -500,42 +500,42 @@
         </is>
       </c>
       <c r="C2" t="n">
-        <v>4131.98</v>
+        <v>3957.05</v>
       </c>
       <c r="D2" t="n">
-        <v>0.09</v>
+        <v>-1.24</v>
       </c>
       <c r="E2" t="n">
-        <v>4104.99</v>
+        <v>4032.26</v>
       </c>
       <c r="F2" t="n">
-        <v>4098.66</v>
+        <v>4073.9</v>
       </c>
       <c r="G2" t="n">
-        <v>4111.41</v>
+        <v>4100.79</v>
       </c>
       <c r="H2" t="n">
-        <v>19.54</v>
+        <v>-20.773</v>
       </c>
       <c r="I2" t="n">
-        <v>24.648</v>
+        <v>-2.47</v>
       </c>
       <c r="J2" t="n">
-        <v>5006852.78</v>
+        <v>6667983.87</v>
       </c>
       <c r="K2" t="n">
-        <v>6998939.76</v>
+        <v>7068821.86</v>
       </c>
       <c r="L2" t="n">
-        <v>0.72</v>
+        <v>0.9399999999999999</v>
       </c>
       <c r="M2" t="inlineStr">
         <is>
-          <t>2026-02-11</t>
+          <t>2026-03-23</t>
         </is>
       </c>
       <c r="N2" t="n">
-        <v>40</v>
+        <v>0</v>
       </c>
     </row>
     <row r="3">
@@ -550,42 +550,42 @@
         </is>
       </c>
       <c r="C3" t="n">
-        <v>14160.93</v>
+        <v>13866.2</v>
       </c>
       <c r="D3" t="n">
-        <v>-0.35</v>
+        <v>-0.25</v>
       </c>
       <c r="E3" t="n">
-        <v>14087.89</v>
+        <v>14060.57</v>
       </c>
       <c r="F3" t="n">
-        <v>14105.31</v>
+        <v>14184.55</v>
       </c>
       <c r="G3" t="n">
-        <v>14205.09</v>
+        <v>14218.97</v>
       </c>
       <c r="H3" t="n">
-        <v>74.718</v>
+        <v>-27.882</v>
       </c>
       <c r="I3" t="n">
-        <v>115.225</v>
+        <v>22.57</v>
       </c>
       <c r="J3" t="n">
-        <v>6819332.01</v>
+        <v>7329346.04</v>
       </c>
       <c r="K3" t="n">
-        <v>8455250.66</v>
+        <v>7663139.2</v>
       </c>
       <c r="L3" t="n">
-        <v>0.8100000000000001</v>
+        <v>0.96</v>
       </c>
       <c r="M3" t="inlineStr">
         <is>
-          <t>2026-02-11</t>
+          <t>2026-03-23</t>
         </is>
       </c>
       <c r="N3" t="n">
-        <v>40</v>
+        <v>0</v>
       </c>
     </row>
     <row r="4">
@@ -600,42 +600,42 @@
         </is>
       </c>
       <c r="C4" t="n">
-        <v>3284.74</v>
+        <v>3352.1</v>
       </c>
       <c r="D4" t="n">
-        <v>-1.08</v>
+        <v>1.3</v>
       </c>
       <c r="E4" t="n">
-        <v>3286.96</v>
+        <v>3328.93</v>
       </c>
       <c r="F4" t="n">
-        <v>3298.62</v>
+        <v>3313.67</v>
       </c>
       <c r="G4" t="n">
-        <v>3314.48</v>
+        <v>3292.26</v>
       </c>
       <c r="H4" t="n">
-        <v>8.856999999999999</v>
+        <v>10.891</v>
       </c>
       <c r="I4" t="n">
-        <v>17.198</v>
+        <v>3.179</v>
       </c>
       <c r="J4" t="n">
-        <v>2207151.23</v>
+        <v>2254016.3</v>
       </c>
       <c r="K4" t="n">
-        <v>2549401.41</v>
+        <v>2303465.08</v>
       </c>
       <c r="L4" t="n">
-        <v>0.87</v>
+        <v>0.98</v>
       </c>
       <c r="M4" t="inlineStr">
         <is>
-          <t>2026-02-11</t>
+          <t>2026-03-23</t>
         </is>
       </c>
       <c r="N4" t="n">
-        <v>40</v>
+        <v>0</v>
       </c>
     </row>
     <row r="5">
@@ -650,42 +650,42 @@
         </is>
       </c>
       <c r="C5" t="n">
-        <v>4713.82</v>
+        <v>4567.02</v>
       </c>
       <c r="D5" t="n">
-        <v>-0.22</v>
+        <v>-0.35</v>
       </c>
       <c r="E5" t="n">
-        <v>4694.24</v>
+        <v>4623.52</v>
       </c>
       <c r="F5" t="n">
-        <v>4689.62</v>
+        <v>4646.9</v>
       </c>
       <c r="G5" t="n">
-        <v>4705.64</v>
+        <v>4665.28</v>
       </c>
       <c r="H5" t="n">
-        <v>4.819</v>
+        <v>-21.085</v>
       </c>
       <c r="I5" t="n">
-        <v>7.236</v>
+        <v>-11.31</v>
       </c>
       <c r="J5" t="n">
-        <v>1733916.81</v>
+        <v>2578737.03</v>
       </c>
       <c r="K5" t="n">
-        <v>2805130.03</v>
+        <v>2742758.71</v>
       </c>
       <c r="L5" t="n">
-        <v>0.62</v>
+        <v>0.9399999999999999</v>
       </c>
       <c r="M5" t="inlineStr">
         <is>
-          <t>2026-02-11</t>
+          <t>2026-03-23</t>
         </is>
       </c>
       <c r="N5" t="n">
-        <v>40</v>
+        <v>0</v>
       </c>
     </row>
   </sheetData>

</xml_diff>